<commit_message>
Added the generation of the output file!
In this state the program is technically functional. But it still requires a few adjustments...
*  Strategic disabling of buttons
   If you have yet to select the source file, or the destination directory, you should not be able to generate press the 'Generate' button.

*  Flexible parsing
   Rn if the input file has any kind of error, the whole thing is halted. It instead would be better if it would carry on, warning in the terminal of the lines that could not be parsed...

*  Completion alert (and terminal use in general)
   It would be great if the program gave you some kind of alert as for when the file is actually generated.
   I mean, it is blazingly fast, but it feels really off that you don't get any cue for that.
   And also, there's the terminal usage to implement, that is for any warning to be displayed there.
</commit_message>
<xml_diff>
--- a/Modelado/Input/Mayores Contables, Modelado Spreadsheet.xlsx
+++ b/Modelado/Input/Mayores Contables, Modelado Spreadsheet.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <bookViews>
-    <workbookView/>
+    <workbookView xWindow="240" yWindow="120" windowWidth="14940" windowHeight="9225" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="1" r:id="rId3"/>
   </sheets>
-  <calcPr fullPrecision="1" calcId="125725"/>
+  <definedNames/>
+  <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="29" count="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
   <si>
     <t>Fecha</t>
   </si>
@@ -82,7 +83,7 @@
     <t>Cierre de Lote Nro.751</t>
   </si>
   <si>
-    <t>Cob Lote Nro. 143 s/Compr.305796</t>
+    <t>Cob. Lote Nro. 143 s/Compr.305796</t>
   </si>
   <si>
     <t>Cob. Lote Nro. 142 s/Compr.305718</t>
@@ -97,7 +98,7 @@
     <t>Cob. Lote Nro. 724 s/Compr.303983</t>
   </si>
   <si>
-    <t>Cierre de Lote Nor.148</t>
+    <t>Cierre de Lote Nro.148</t>
   </si>
   <si>
     <t>Totales:</t>
@@ -106,46 +107,26 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none">
-        <fgColor indexed="64"/>
-        <bgColor indexed="65"/>
-      </patternFill>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125">
-        <fgColor indexed="64"/>
-        <bgColor indexed="65"/>
-      </patternFill>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
@@ -157,66 +138,444 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="26">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyNumberFormat="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
+      <protection/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment/>
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="Hoja1LockedColumnStyle" xfId="20"/>
-    <cellStyle name="Hoja1UnLockedColumnStyle" xfId="21"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="3" builtinId="7"/>
+    <cellStyle name="Comma" xfId="4" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="5" builtinId="6"/>
+    <cellStyle name="Hoja1LockedColumnStyle" xfId="6"/>
+    <cellStyle name="Hoja1UnLockedColumnStyle" xfId="7"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="44546A"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E7E6E6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4472C4"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="ED7D31"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A5A5A5"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="FFC000"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="5B9BD5"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="70AD47"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0563C1"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="954F72"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F27"/>
-  <sheetFormatPr customHeight="true" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="3" max="3" width="32.41796875" customWidth="1"/>
-    <col min="4" max="6" width="11.41796875" customWidth="1"/>
+    <col min="3" max="3" width="32.4285714285714" customWidth="1"/>
+    <col min="4" max="6" width="11.4285714285714" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" ht="15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -236,7 +595,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" ht="15">
       <c r="A2" s="2">
         <v>46023</v>
       </c>
@@ -254,7 +613,7 @@
         <v>19912.12</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" ht="15">
       <c r="A3" s="2">
         <v>46026</v>
       </c>
@@ -272,7 +631,7 @@
         <v>20212.12</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" ht="15">
       <c r="A4" s="2">
         <v>46027</v>
       </c>
@@ -290,7 +649,7 @@
         <v>20412.12</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" ht="15">
       <c r="A5" s="2">
         <v>46027</v>
       </c>
@@ -308,7 +667,7 @@
         <v>10487.12</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" ht="15">
       <c r="A6" s="2">
         <v>46028</v>
       </c>
@@ -326,7 +685,7 @@
         <v>10687.12</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" ht="15">
       <c r="A7" s="2">
         <v>46029</v>
       </c>
@@ -344,7 +703,7 @@
         <v>10387.12</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" ht="15">
       <c r="A8" s="2">
         <v>46029</v>
       </c>
@@ -362,7 +721,7 @@
         <v>10187.12</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" ht="15">
       <c r="A9" s="2">
         <v>46030</v>
       </c>
@@ -380,7 +739,7 @@
         <v>10487.12</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" ht="15">
       <c r="A10" s="2">
         <v>46030</v>
       </c>
@@ -398,7 +757,7 @@
         <v>10287.12</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" ht="15">
       <c r="A11" s="2">
         <v>46031</v>
       </c>
@@ -416,7 +775,7 @@
         <v>10407.12</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" ht="15">
       <c r="A12" s="2">
         <v>46031</v>
       </c>
@@ -434,7 +793,7 @@
         <v>8007.12</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" ht="15">
       <c r="A13" s="2">
         <v>46031</v>
       </c>
@@ -452,7 +811,7 @@
         <v>5607.12</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" ht="15">
       <c r="A14" s="2">
         <v>46031</v>
       </c>
@@ -470,7 +829,7 @@
         <v>3207.12</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" ht="15">
       <c r="A15" s="2">
         <v>46031</v>
       </c>
@@ -488,7 +847,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" ht="15">
       <c r="A16" s="2">
         <v>46032</v>
       </c>
@@ -506,7 +865,7 @@
         <v>10217.12</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" ht="15">
       <c r="A17" s="2">
         <v>46032</v>
       </c>
@@ -524,7 +883,7 @@
         <v>17142.12</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" ht="15">
       <c r="A18" s="2">
         <v>46032</v>
       </c>
@@ -542,7 +901,7 @@
         <v>30992.12</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" ht="15">
       <c r="A19" s="2">
         <v>46032</v>
       </c>
@@ -560,7 +919,7 @@
         <v>31092.12</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" ht="15">
       <c r="A20" s="2">
         <v>46034</v>
       </c>
@@ -578,7 +937,7 @@
         <v>31392.12</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" ht="15">
       <c r="A21" s="2">
         <v>46035</v>
       </c>
@@ -596,7 +955,7 @@
         <v>17542.12</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" ht="15">
       <c r="A22" s="2">
         <v>46035</v>
       </c>
@@ -614,7 +973,7 @@
         <v>10617.12</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" ht="15">
       <c r="A23" s="2">
         <v>46035</v>
       </c>
@@ -632,7 +991,7 @@
         <v>10317.12</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" ht="15">
       <c r="A24" s="2">
         <v>46036</v>
       </c>
@@ -650,7 +1009,7 @@
         <v>10117.12</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" ht="15">
       <c r="A25" s="2">
         <v>46036</v>
       </c>
@@ -668,7 +1027,7 @@
         <v>9817.12</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" ht="15">
       <c r="A26" s="2">
         <v>46037</v>
       </c>
@@ -686,7 +1045,7 @@
         <v>15317.12</v>
       </c>
     </row>
-    <row r="27" spans="4:6">
+    <row r="27" spans="4:6" ht="15">
       <c r="D27" s="1" t="s">
         <v>28</v>
       </c>
@@ -699,7 +1058,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter scaleWithDoc="1" alignWithMargins="0" differentFirst="0" differentOddEven="0"/>
-  <extLst/>
+  <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
</xml_diff>